<commit_message>
Move Big Plasmid Box
</commit_message>
<xml_diff>
--- a/cellstocks/data/baris.xlsx
+++ b/cellstocks/data/baris.xlsx
@@ -57436,12 +57436,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Big Plasmid Box</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -57468,17 +57468,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fridge 1</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ChIP Box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -57515,7 +57515,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">ChIP Box -2-</t>
+          <t xml:space="preserve">ChIP Box</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -57552,7 +57552,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Umut -20 -2-</t>
+          <t xml:space="preserve">ChIP Box -2-</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -57589,7 +57589,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Umut -20 Box -1-</t>
+          <t xml:space="preserve">Umut -20 -2-</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -57616,17 +57616,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Fridge 1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unkown FOR NOW</t>
+          <t xml:space="preserve">Umut -20 Box -1-</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -57663,7 +57663,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">No use</t>
+          <t xml:space="preserve">Unkown FOR NOW</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -57700,7 +57700,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Big Plasmid Box</t>
+          <t xml:space="preserve">No use</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">

</xml_diff>